<commit_message>
Added docs for 2 new endpoints for viewing categories
</commit_message>
<xml_diff>
--- a/docs/api_endpoints.xlsx
+++ b/docs/api_endpoints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dmoreland/projects/soa-workbench/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2013FAE1-3D34-E448-A2E4-A787FE83D7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6BE5E82-94D4-3645-B442-B672F8B58515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1340" yWindow="1880" windowWidth="32920" windowHeight="17180" xr2:uid="{9BDE69E9-CFA3-1D4B-8A38-383A8A36D10D}"/>
+    <workbookView xWindow="-21600" yWindow="10240" windowWidth="21600" windowHeight="17180" xr2:uid="{9BDE69E9-CFA3-1D4B-8A38-383A8A36D10D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="183">
   <si>
     <t>Method</t>
   </si>
@@ -655,7 +655,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -664,16 +664,10 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -681,6 +675,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1016,14 +1013,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C63BF3E0-94E9-7C4C-9734-A7F780535720}">
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="55.1640625" customWidth="1"/>
     <col min="2" max="2" width="24.5" customWidth="1"/>
     <col min="3" max="3" width="42.5" customWidth="1"/>
     <col min="4" max="4" width="43.6640625" customWidth="1"/>
-    <col min="5" max="5" width="48.5" style="9" customWidth="1"/>
+    <col min="5" max="5" width="48.5" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="20" x14ac:dyDescent="0.2">
@@ -1039,7 +1036,7 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1056,7 +1053,7 @@
       <c r="D2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>136</v>
       </c>
     </row>
@@ -1073,7 +1070,7 @@
       <c r="D3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>167</v>
       </c>
     </row>
@@ -1090,7 +1087,7 @@
       <c r="D4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>175</v>
       </c>
     </row>
@@ -1107,7 +1104,7 @@
       <c r="D5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1124,7 +1121,7 @@
       <c r="D6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>168</v>
       </c>
     </row>
@@ -1141,7 +1138,7 @@
       <c r="D7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>171</v>
       </c>
     </row>
@@ -1158,7 +1155,7 @@
       <c r="D8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>172</v>
       </c>
     </row>
@@ -1175,7 +1172,7 @@
       <c r="D9" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>173</v>
       </c>
     </row>
@@ -1192,7 +1189,7 @@
       <c r="D10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>176</v>
       </c>
     </row>
@@ -1209,7 +1206,7 @@
       <c r="D11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>182</v>
       </c>
     </row>
@@ -1226,7 +1223,7 @@
       <c r="D12" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>179</v>
       </c>
     </row>
@@ -1243,7 +1240,7 @@
       <c r="D13" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>180</v>
       </c>
     </row>
@@ -1260,7 +1257,7 @@
       <c r="D14" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1277,7 +1274,7 @@
       <c r="D15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1294,7 +1291,7 @@
       <c r="D16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="5" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1311,7 +1308,7 @@
       <c r="D17" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E17" s="6"/>
+      <c r="E17" s="5"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
@@ -1326,7 +1323,7 @@
       <c r="D18" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E18" s="6"/>
+      <c r="E18" s="5"/>
     </row>
     <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
@@ -1341,7 +1338,7 @@
       <c r="D19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="5" t="s">
         <v>134</v>
       </c>
     </row>
@@ -1358,7 +1355,7 @@
       <c r="D20" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="6"/>
+      <c r="E20" s="5"/>
     </row>
     <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -1373,7 +1370,7 @@
       <c r="D21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="5" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1390,7 +1387,7 @@
       <c r="D22" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="6"/>
+      <c r="E22" s="5"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -1405,7 +1402,7 @@
       <c r="D23" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E23" s="6"/>
+      <c r="E23" s="5"/>
     </row>
     <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
@@ -1420,7 +1417,7 @@
       <c r="D24" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="5" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1437,7 +1434,7 @@
       <c r="D25" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="E25" s="6"/>
+      <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
@@ -1452,7 +1449,7 @@
       <c r="D26" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E26" s="6"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
@@ -1467,7 +1464,7 @@
       <c r="D27" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E27" s="6"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
@@ -1482,7 +1479,7 @@
       <c r="D28" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E28" s="6"/>
+      <c r="E28" s="5"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
@@ -1497,7 +1494,7 @@
       <c r="D29" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="E29" s="6"/>
+      <c r="E29" s="5"/>
     </row>
     <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
@@ -1512,7 +1509,7 @@
       <c r="D30" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="5" t="s">
         <v>128</v>
       </c>
     </row>
@@ -1529,7 +1526,7 @@
       <c r="D31" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E31" s="6"/>
+      <c r="E31" s="5"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
@@ -1544,7 +1541,7 @@
       <c r="D32" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E32" s="6"/>
+      <c r="E32" s="5"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
@@ -1559,7 +1556,7 @@
       <c r="D33" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E33" s="6"/>
+      <c r="E33" s="5"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
@@ -1574,7 +1571,7 @@
       <c r="D34" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E34" s="6"/>
+      <c r="E34" s="5"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
@@ -1589,7 +1586,7 @@
       <c r="D35" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E35" s="6"/>
+      <c r="E35" s="5"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
@@ -1604,7 +1601,7 @@
       <c r="D36" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E36" s="6"/>
+      <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
@@ -1619,7 +1616,7 @@
       <c r="D37" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E37" s="6"/>
+      <c r="E37" s="5"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
@@ -1634,7 +1631,7 @@
       <c r="D38" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E38" s="6"/>
+      <c r="E38" s="5"/>
     </row>
     <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
@@ -1649,7 +1646,7 @@
       <c r="D39" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="E39" s="5" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1666,7 +1663,7 @@
       <c r="D40" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E40" s="6"/>
+      <c r="E40" s="5"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
@@ -1681,7 +1678,7 @@
       <c r="D41" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E41" s="6"/>
+      <c r="E41" s="5"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
@@ -1696,7 +1693,7 @@
       <c r="D42" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="E42" s="6"/>
+      <c r="E42" s="5"/>
     </row>
     <row r="43" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
@@ -1711,7 +1708,7 @@
       <c r="D43" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="E43" s="5" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1728,7 +1725,7 @@
       <c r="D44" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="E44" s="5" t="s">
         <v>130</v>
       </c>
     </row>
@@ -1745,7 +1742,7 @@
       <c r="D45" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E45" s="6"/>
+      <c r="E45" s="5"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
@@ -1760,7 +1757,7 @@
       <c r="D46" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E46" s="6"/>
+      <c r="E46" s="5"/>
     </row>
     <row r="47" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
@@ -1775,7 +1772,7 @@
       <c r="D47" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="E47" s="5" t="s">
         <v>129</v>
       </c>
     </row>
@@ -1792,7 +1789,7 @@
       <c r="D48" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="E48" s="5" t="s">
         <v>132</v>
       </c>
     </row>
@@ -1809,7 +1806,7 @@
       <c r="D49" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E49" s="5" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1826,7 +1823,7 @@
       <c r="D50" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E50" s="6"/>
+      <c r="E50" s="5"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
@@ -1841,7 +1838,7 @@
       <c r="D51" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E51" s="6"/>
+      <c r="E51" s="5"/>
     </row>
     <row r="52" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
@@ -1856,7 +1853,7 @@
       <c r="D52" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E52" s="6" t="s">
+      <c r="E52" s="5" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1873,7 +1870,7 @@
       <c r="D53" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E53" s="6"/>
+      <c r="E53" s="5"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
@@ -1888,7 +1885,7 @@
       <c r="D54" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E54" s="6"/>
+      <c r="E54" s="5"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
@@ -1903,7 +1900,7 @@
       <c r="D55" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E55" s="6"/>
+      <c r="E55" s="5"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
@@ -1918,7 +1915,7 @@
       <c r="D56" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E56" s="6"/>
+      <c r="E56" s="5"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
@@ -1933,7 +1930,7 @@
       <c r="D57" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E57" s="6"/>
+      <c r="E57" s="5"/>
     </row>
     <row r="58" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
@@ -1948,7 +1945,7 @@
       <c r="D58" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E58" s="6" t="s">
+      <c r="E58" s="5" t="s">
         <v>133</v>
       </c>
     </row>
@@ -1965,7 +1962,7 @@
       <c r="D59" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E59" s="6"/>
+      <c r="E59" s="5"/>
     </row>
     <row r="60" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
@@ -1980,7 +1977,7 @@
       <c r="D60" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E60" s="6" t="s">
+      <c r="E60" s="5" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1997,7 +1994,7 @@
       <c r="D61" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E61" s="6"/>
+      <c r="E61" s="5"/>
     </row>
     <row r="62" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
@@ -2006,13 +2003,13 @@
       <c r="B62" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C62" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E62" s="7" t="s">
+      <c r="C62" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E62" s="5" t="s">
         <v>110</v>
       </c>
     </row>
@@ -2023,13 +2020,13 @@
       <c r="B63" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C63" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E63" s="8" t="s">
+      <c r="C63" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2046,7 +2043,7 @@
       <c r="D64" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E64" s="6" t="s">
+      <c r="E64" s="5" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2063,7 +2060,7 @@
       <c r="D65" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E65" s="6" t="s">
+      <c r="E65" s="5" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2080,7 +2077,7 @@
       <c r="D66" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E66" s="6" t="s">
+      <c r="E66" s="5" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2097,7 +2094,7 @@
       <c r="D67" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E67" s="6" t="s">
+      <c r="E67" s="5" t="s">
         <v>174</v>
       </c>
     </row>
@@ -2114,7 +2111,7 @@
       <c r="D68" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="E68" s="5" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2131,7 +2128,7 @@
       <c r="D69" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E69" s="6" t="s">
+      <c r="E69" s="5" t="s">
         <v>177</v>
       </c>
     </row>
@@ -2148,7 +2145,7 @@
       <c r="D70" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E70" s="6" t="s">
+      <c r="E70" s="5" t="s">
         <v>181</v>
       </c>
     </row>
@@ -2165,7 +2162,7 @@
       <c r="D71" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E71" s="6" t="s">
+      <c r="E71" s="5" t="s">
         <v>178</v>
       </c>
     </row>
@@ -2182,7 +2179,7 @@
       <c r="D72" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E72" s="6" t="s">
+      <c r="E72" s="5" t="s">
         <v>142</v>
       </c>
     </row>
@@ -2199,7 +2196,7 @@
       <c r="D73" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E73" s="6" t="s">
+      <c r="E73" s="5" t="s">
         <v>143</v>
       </c>
     </row>
@@ -2216,7 +2213,7 @@
       <c r="D74" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E74" s="6" t="s">
+      <c r="E74" s="5" t="s">
         <v>118</v>
       </c>
     </row>
@@ -2233,7 +2230,7 @@
       <c r="D75" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E75" s="6" t="s">
+      <c r="E75" s="5" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2250,7 +2247,7 @@
       <c r="D76" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E76" s="6" t="s">
+      <c r="E76" s="5" t="s">
         <v>154</v>
       </c>
     </row>
@@ -2267,7 +2264,7 @@
       <c r="D77" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E77" s="6" t="s">
+      <c r="E77" s="5" t="s">
         <v>157</v>
       </c>
     </row>
@@ -2284,7 +2281,7 @@
       <c r="D78" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E78" s="6" t="s">
+      <c r="E78" s="5" t="s">
         <v>125</v>
       </c>
     </row>
@@ -2301,7 +2298,7 @@
       <c r="D79" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E79" s="6" t="s">
+      <c r="E79" s="5" t="s">
         <v>127</v>
       </c>
     </row>
@@ -2318,7 +2315,7 @@
       <c r="D80" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E80" s="6" t="s">
+      <c r="E80" s="5" t="s">
         <v>137</v>
       </c>
     </row>
@@ -2335,7 +2332,7 @@
       <c r="D81" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E81" s="6" t="s">
+      <c r="E81" s="5" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2352,7 +2349,7 @@
       <c r="D82" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E82" s="6" t="s">
+      <c r="E82" s="5" t="s">
         <v>149</v>
       </c>
     </row>
@@ -2369,7 +2366,7 @@
       <c r="D83" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E83" s="6" t="s">
+      <c r="E83" s="5" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2386,7 +2383,7 @@
       <c r="D84" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E84" s="6" t="s">
+      <c r="E84" s="5" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2403,7 +2400,7 @@
       <c r="D85" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E85" s="6" t="s">
+      <c r="E85" s="5" t="s">
         <v>119</v>
       </c>
     </row>
@@ -2420,7 +2417,7 @@
       <c r="D86" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E86" s="6" t="s">
+      <c r="E86" s="5" t="s">
         <v>162</v>
       </c>
     </row>
@@ -2437,7 +2434,7 @@
       <c r="D87" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E87" s="6"/>
+      <c r="E87" s="5"/>
     </row>
     <row r="88" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
@@ -2452,7 +2449,7 @@
       <c r="D88" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E88" s="6" t="s">
+      <c r="E88" s="5" t="s">
         <v>151</v>
       </c>
     </row>
@@ -2469,7 +2466,7 @@
       <c r="D89" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E89" s="6" t="s">
+      <c r="E89" s="5" t="s">
         <v>163</v>
       </c>
     </row>
@@ -2486,7 +2483,7 @@
       <c r="D90" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E90" s="6" t="s">
+      <c r="E90" s="5" t="s">
         <v>160</v>
       </c>
     </row>
@@ -2503,7 +2500,7 @@
       <c r="D91" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E91" s="6" t="s">
+      <c r="E91" s="5" t="s">
         <v>140</v>
       </c>
     </row>
@@ -2520,7 +2517,7 @@
       <c r="D92" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E92" s="6"/>
+      <c r="E92" s="5"/>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
@@ -2535,7 +2532,7 @@
       <c r="D93" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E93" s="6"/>
+      <c r="E93" s="5"/>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
@@ -2550,7 +2547,7 @@
       <c r="D94" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E94" s="6"/>
+      <c r="E94" s="5"/>
     </row>
     <row r="95" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
@@ -2565,7 +2562,7 @@
       <c r="D95" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E95" s="6" t="s">
+      <c r="E95" s="5" t="s">
         <v>165</v>
       </c>
     </row>
@@ -2582,7 +2579,7 @@
       <c r="D96" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E96" s="6" t="s">
+      <c r="E96" s="5" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2599,7 +2596,7 @@
       <c r="D97" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E97" s="6"/>
+      <c r="E97" s="5"/>
     </row>
     <row r="98" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
@@ -2614,7 +2611,7 @@
       <c r="D98" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E98" s="6" t="s">
+      <c r="E98" s="5" t="s">
         <v>166</v>
       </c>
     </row>
@@ -2631,7 +2628,7 @@
       <c r="D99" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E99" s="6" t="s">
+      <c r="E99" s="5" t="s">
         <v>164</v>
       </c>
     </row>
@@ -2648,7 +2645,7 @@
       <c r="D100" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="E100" s="6"/>
+      <c r="E100" s="5"/>
     </row>
     <row r="101" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
@@ -2663,7 +2660,7 @@
       <c r="D101" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E101" s="6" t="s">
+      <c r="E101" s="5" t="s">
         <v>158</v>
       </c>
     </row>
@@ -2680,7 +2677,7 @@
       <c r="D102" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E102" s="6" t="s">
+      <c r="E102" s="5" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2697,7 +2694,7 @@
       <c r="D103" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E103" s="6" t="s">
+      <c r="E103" s="5" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2714,7 +2711,7 @@
       <c r="D104" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E104" s="6" t="s">
+      <c r="E104" s="5" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2731,7 +2728,7 @@
       <c r="D105" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E105" s="6" t="s">
+      <c r="E105" s="5" t="s">
         <v>150</v>
       </c>
     </row>
@@ -2748,7 +2745,7 @@
       <c r="D106" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E106" s="6" t="s">
+      <c r="E106" s="5" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2765,7 +2762,7 @@
       <c r="D107" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E107" s="6" t="s">
+      <c r="E107" s="5" t="s">
         <v>139</v>
       </c>
     </row>
@@ -2782,8 +2779,42 @@
       <c r="D108" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E108" s="6" t="s">
+      <c r="E108" s="5" t="s">
         <v>138</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A109" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B109" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C109" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D109" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E109" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A110" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D110" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E110" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>